<commit_message>
DB - Update 1.1
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -1275,25 +1275,19 @@
           <t>Entropiq</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G23" t="n">
+        <v>8</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1812,14 +1806,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" t="n">
-        <v>-5</v>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -4314,20 +4314,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E103" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" t="n">
+        <v>-5</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -4575,19 +4569,25 @@
           <t>hoorai</t>
         </is>
       </c>
-      <c r="D110" t="n">
-        <v>1</v>
-      </c>
-      <c r="E110" t="n">
-        <v>1</v>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G110" t="n">
-        <v>8</v>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
update 1.0 (americas oq)
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -479,12 +479,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -517,7 +517,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -527,12 +527,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>-12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -555,22 +555,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -631,22 +631,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -717,12 +717,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -755,12 +755,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -897,22 +897,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -935,17 +935,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -973,22 +973,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1021,12 +1021,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1059,12 +1059,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1097,12 +1097,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1211,12 +1211,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1239,12 +1239,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1277,12 +1277,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1325,12 +1325,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1363,12 +1363,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1401,12 +1401,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1541,25 +1541,19 @@
           <t>SK</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>8</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1584,20 +1578,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>-5</t>
-        </is>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-5</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1657,22 +1645,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1705,12 +1693,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1743,12 +1731,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1771,7 +1759,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1781,12 +1769,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>-12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1819,12 +1807,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1847,7 +1835,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1857,12 +1845,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1895,12 +1883,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1933,12 +1921,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1971,12 +1959,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2009,12 +1997,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2037,7 +2025,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2047,12 +2035,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>-4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2075,22 +2063,22 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2113,22 +2101,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2161,12 +2149,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2199,12 +2187,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2263,25 +2251,19 @@
           <t>M80</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>8</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2303,7 +2285,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2313,12 +2295,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>-12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2341,12 +2323,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2356,7 +2338,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2377,25 +2359,19 @@
           <t>ECSTATIC</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>-4</t>
-        </is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>8</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2415,25 +2391,19 @@
           <t>RED Canids</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>8</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2531,22 +2501,22 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
           <t>8</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>51</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2579,12 +2549,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2607,7 +2577,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2617,12 +2587,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>-3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2683,22 +2653,22 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2731,12 +2701,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2759,12 +2729,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2774,7 +2744,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -2797,12 +2767,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2812,7 +2782,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -2876,20 +2846,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>-5</t>
-        </is>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-5</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -2921,12 +2885,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -2959,12 +2923,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -2987,7 +2951,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2997,12 +2961,12 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3025,22 +2989,22 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3073,12 +3037,12 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3101,12 +3065,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3116,7 +3080,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3149,12 +3113,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3177,22 +3141,22 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3225,12 +3189,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3253,12 +3217,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3268,7 +3232,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3301,12 +3265,12 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3329,12 +3293,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3344,7 +3308,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3367,12 +3331,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3382,7 +3346,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3415,12 +3379,12 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3441,17 +3405,25 @@
           <t>NAVI Junior</t>
         </is>
       </c>
-      <c r="D80" t="n">
-        <v>7</v>
-      </c>
-      <c r="E80" t="n">
-        <v>1</v>
-      </c>
-      <c r="F80" t="n">
-        <v>1</v>
-      </c>
-      <c r="G80" t="n">
-        <v>66</v>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -3483,12 +3455,12 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3521,12 +3493,12 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3549,12 +3521,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3564,7 +3536,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3597,12 +3569,12 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -3635,12 +3607,12 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -3663,12 +3635,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3678,7 +3650,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -3711,12 +3683,12 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -3742,20 +3714,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>-5</t>
-        </is>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" t="n">
+        <v>-5</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -3777,12 +3743,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3792,7 +3758,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -3825,12 +3791,12 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -3863,12 +3829,12 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -3891,12 +3857,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3906,7 +3872,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -3939,12 +3905,12 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -3967,7 +3933,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -3977,7 +3943,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4005,12 +3971,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4020,7 +3986,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4053,12 +4019,12 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4091,12 +4057,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4119,12 +4085,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4134,7 +4100,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4167,12 +4133,12 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4205,12 +4171,12 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4231,17 +4197,25 @@
           <t>Onyx Ravens</t>
         </is>
       </c>
-      <c r="D101" t="n">
-        <v>4</v>
-      </c>
-      <c r="E101" t="n">
-        <v>0</v>
-      </c>
-      <c r="F101" t="n">
-        <v>3</v>
-      </c>
-      <c r="G101" t="n">
-        <v>18</v>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -4273,12 +4247,12 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4311,12 +4285,12 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4339,22 +4313,22 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4377,22 +4351,22 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -4418,20 +4392,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>-5</t>
-        </is>
+      <c r="E106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" t="n">
+        <v>-5</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -4463,12 +4431,12 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -4529,22 +4497,22 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -4567,12 +4535,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -4582,7 +4550,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -4605,22 +4573,22 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -4643,22 +4611,22 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -4995,12 +4963,12 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">

</xml_diff>

<commit_message>
update 2.0 (europe oq)
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -479,12 +479,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -515,25 +515,19 @@
           <t>Astralis</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G3" t="n">
+        <v>8</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -631,12 +625,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -646,7 +640,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -707,12 +701,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -722,7 +716,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -755,12 +749,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -781,25 +775,19 @@
           <t>ENCE</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G10" t="n">
+        <v>8</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -831,12 +819,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1014,20 +1002,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-5</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1047,25 +1029,19 @@
           <t>G2</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G17" t="n">
+        <v>8</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1087,12 +1063,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1102,7 +1078,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1315,12 +1291,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1330,7 +1306,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1363,12 +1339,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1389,25 +1365,19 @@
           <t>iBUYPOWER</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G26" t="n">
+        <v>8</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1470,20 +1440,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-5</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1505,12 +1469,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1520,7 +1484,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1541,19 +1505,25 @@
           <t>SK</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" t="n">
-        <v>1</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G30" t="n">
-        <v>8</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1578,14 +1548,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" t="n">
-        <v>-5</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1686,20 +1662,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-5</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1757,25 +1727,19 @@
           <t>ShindeN</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G36" t="n">
+        <v>8</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -1835,12 +1799,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1850,7 +1814,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1921,12 +1885,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1952,20 +1916,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-5</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2023,25 +1981,19 @@
           <t>Permitta</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G43" t="n">
+        <v>8</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2061,25 +2013,19 @@
           <t>Rebels</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G44" t="n">
+        <v>8</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2099,25 +2045,19 @@
           <t>Eternal Fire</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G45" t="n">
+        <v>8</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2142,20 +2082,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-5</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2180,20 +2114,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-5</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2251,19 +2179,25 @@
           <t>M80</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" t="n">
-        <v>1</v>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G49" t="n">
-        <v>8</v>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2285,12 +2219,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2300,7 +2234,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2359,19 +2293,25 @@
           <t>ECSTATIC</t>
         </is>
       </c>
-      <c r="D52" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" t="n">
-        <v>1</v>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G52" t="n">
-        <v>8</v>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2391,19 +2331,25 @@
           <t>RED Canids</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" t="n">
-        <v>1</v>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G53" t="n">
-        <v>8</v>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2549,12 +2495,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2701,12 +2647,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2846,14 +2792,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E65" t="n">
-        <v>0</v>
-      </c>
-      <c r="F65" t="n">
-        <v>1</v>
-      </c>
-      <c r="G65" t="n">
-        <v>-5</v>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -3037,12 +2989,12 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3189,12 +3141,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3714,14 +3666,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E88" t="n">
-        <v>0</v>
-      </c>
-      <c r="F88" t="n">
-        <v>1</v>
-      </c>
-      <c r="G88" t="n">
-        <v>-5</v>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -4392,14 +4350,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E106" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" t="n">
-        <v>1</v>
-      </c>
-      <c r="G106" t="n">
-        <v>-5</v>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -4416,7 +4380,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>LCDC</t>
+          <t>LDLC</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -4424,20 +4388,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" t="n">
+        <v>-5</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -4956,20 +4914,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E121" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" t="n">
+        <v>1</v>
+      </c>
+      <c r="G121" t="n">
+        <v>-5</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
update 3.0 (asia oq)
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -515,19 +515,25 @@
           <t>Astralis</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>8</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -775,19 +781,25 @@
           <t>ENCE</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>8</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -961,12 +973,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -976,7 +988,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1002,14 +1014,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
-        <v>-5</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1029,19 +1047,25 @@
           <t>G2</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G17" t="n">
-        <v>8</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1177,12 +1201,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1192,7 +1216,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1215,12 +1239,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1230,7 +1254,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1251,25 +1275,19 @@
           <t>Entropiq</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G23" t="n">
+        <v>8</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1365,19 +1383,25 @@
           <t>iBUYPOWER</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="n">
-        <v>1</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G26" t="n">
-        <v>8</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1409,12 +1433,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1440,14 +1464,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" t="n">
-        <v>-5</v>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1662,14 +1692,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" t="n">
-        <v>-5</v>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1701,12 +1737,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1727,19 +1763,25 @@
           <t>ShindeN</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" t="n">
-        <v>1</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G36" t="n">
-        <v>8</v>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -1764,20 +1806,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-5</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -1847,12 +1883,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1916,14 +1952,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E41" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" t="n">
-        <v>-5</v>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -1955,12 +1997,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -1981,19 +2023,25 @@
           <t>Permitta</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" t="n">
-        <v>1</v>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G43" t="n">
-        <v>8</v>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2013,19 +2061,25 @@
           <t>Rebels</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" t="n">
-        <v>1</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G44" t="n">
-        <v>8</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2045,19 +2099,25 @@
           <t>Eternal Fire</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" t="n">
-        <v>1</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G45" t="n">
-        <v>8</v>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2082,14 +2142,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" t="n">
-        <v>-5</v>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2114,14 +2180,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E47" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" t="n">
-        <v>-5</v>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2257,12 +2329,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2272,7 +2344,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2521,25 +2593,19 @@
           <t>Underground</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G58" t="n">
+        <v>8</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -2673,25 +2739,19 @@
           <t>Homyno</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G62" t="n">
+        <v>8</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -2713,12 +2773,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2728,7 +2788,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -2837,12 +2897,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -2875,12 +2935,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -2903,12 +2963,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2918,7 +2978,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3017,12 +3077,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3032,7 +3092,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3065,12 +3125,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3091,25 +3151,19 @@
           <t>The MongolZ</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G73" t="n">
+        <v>8</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -3169,12 +3223,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3184,7 +3238,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3217,12 +3271,12 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3245,12 +3299,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3260,7 +3314,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3283,12 +3337,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3298,7 +3352,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3324,20 +3378,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-5</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -3359,12 +3407,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3374,7 +3422,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3407,12 +3455,12 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3445,12 +3493,12 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3471,25 +3519,19 @@
           <t>TYLOO</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G83" t="n">
+        <v>8</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -3521,12 +3563,12 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -3552,20 +3594,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" t="n">
+        <v>-5</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -3587,12 +3623,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3602,7 +3638,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -3635,12 +3671,12 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -3699,25 +3735,19 @@
           <t>MenaceGG</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G89" t="n">
+        <v>8</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -3742,20 +3772,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" t="n">
+        <v>-5</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -3780,20 +3804,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" t="n">
+        <v>-5</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -3815,12 +3833,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3830,7 +3848,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -3863,12 +3881,12 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -3889,25 +3907,19 @@
           <t>True Rippers</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" t="n">
+        <v>1</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G94" t="n">
+        <v>8</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -3929,12 +3941,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -3944,7 +3956,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -3977,12 +3989,12 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4015,12 +4027,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4043,12 +4055,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4058,7 +4070,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4084,20 +4096,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" t="n">
+        <v>-5</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -4122,20 +4128,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
+      </c>
+      <c r="G100" t="n">
+        <v>-5</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -4157,12 +4157,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -4205,12 +4205,12 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4236,20 +4236,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E103" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" t="n">
+        <v>-5</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -4388,14 +4382,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E107" t="n">
-        <v>0</v>
-      </c>
-      <c r="F107" t="n">
-        <v>1</v>
-      </c>
-      <c r="G107" t="n">
-        <v>-5</v>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -4491,25 +4491,19 @@
           <t>hoorai</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D110" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" t="n">
+        <v>1</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="G110" t="n">
+        <v>8</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -4914,14 +4908,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E121" t="n">
-        <v>0</v>
-      </c>
-      <c r="F121" t="n">
-        <v>1</v>
-      </c>
-      <c r="G121" t="n">
-        <v>-5</v>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
update 3.1 (americas rmr a)
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -895,25 +895,17 @@
           <t>Legacy</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>5</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1275,19 +1267,25 @@
           <t>Entropiq</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" t="n">
-        <v>1</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G23" t="n">
-        <v>8</v>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1649,25 +1647,19 @@
           <t>Iluminar</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D33" t="n">
+        <v>7</v>
+      </c>
+      <c r="E33" t="n">
+        <v>6</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>66</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -1806,14 +1798,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" t="n">
-        <v>-5</v>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2253,23 +2251,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>4</v>
+      </c>
+      <c r="G49" t="n">
+        <v>7</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2403,25 +2395,17 @@
           <t>RED Canids</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D53" t="n">
+        <v>5</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>4</v>
+      </c>
+      <c r="G53" t="n">
+        <v>24</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2593,19 +2577,25 @@
           <t>Underground</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" t="n">
-        <v>1</v>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G58" t="n">
-        <v>8</v>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -2739,19 +2729,25 @@
           <t>Homyno</t>
         </is>
       </c>
-      <c r="D62" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" t="n">
-        <v>1</v>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G62" t="n">
-        <v>8</v>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -3151,19 +3147,25 @@
           <t>The MongolZ</t>
         </is>
       </c>
-      <c r="D73" t="n">
-        <v>1</v>
-      </c>
-      <c r="E73" t="n">
-        <v>1</v>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G73" t="n">
-        <v>8</v>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -3378,14 +3380,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E79" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" t="n">
-        <v>1</v>
-      </c>
-      <c r="G79" t="n">
-        <v>-5</v>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -3519,19 +3527,25 @@
           <t>TYLOO</t>
         </is>
       </c>
-      <c r="D83" t="n">
-        <v>1</v>
-      </c>
-      <c r="E83" t="n">
-        <v>1</v>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G83" t="n">
-        <v>8</v>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -3594,14 +3608,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E85" t="n">
-        <v>0</v>
-      </c>
-      <c r="F85" t="n">
-        <v>1</v>
-      </c>
-      <c r="G85" t="n">
-        <v>-5</v>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -3735,19 +3755,25 @@
           <t>MenaceGG</t>
         </is>
       </c>
-      <c r="D89" t="n">
-        <v>1</v>
-      </c>
-      <c r="E89" t="n">
-        <v>1</v>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G89" t="n">
-        <v>8</v>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -3772,14 +3798,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E90" t="n">
-        <v>0</v>
-      </c>
-      <c r="F90" t="n">
-        <v>1</v>
-      </c>
-      <c r="G90" t="n">
-        <v>-5</v>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -3804,14 +3836,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F91" t="n">
-        <v>1</v>
-      </c>
-      <c r="G91" t="n">
-        <v>-5</v>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -3907,19 +3945,25 @@
           <t>True Rippers</t>
         </is>
       </c>
-      <c r="D94" t="n">
-        <v>1</v>
-      </c>
-      <c r="E94" t="n">
-        <v>1</v>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G94" t="n">
-        <v>8</v>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -4096,14 +4140,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E99" t="n">
-        <v>0</v>
-      </c>
-      <c r="F99" t="n">
-        <v>1</v>
-      </c>
-      <c r="G99" t="n">
-        <v>-5</v>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -4128,14 +4178,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E100" t="n">
-        <v>0</v>
-      </c>
-      <c r="F100" t="n">
-        <v>1</v>
-      </c>
-      <c r="G100" t="n">
-        <v>-5</v>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -4236,14 +4292,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E103" t="n">
-        <v>0</v>
-      </c>
-      <c r="F103" t="n">
-        <v>1</v>
-      </c>
-      <c r="G103" t="n">
-        <v>-5</v>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -4263,25 +4325,17 @@
           <t>Bad News Eagles</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D104" t="n">
+        <v>3</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" t="n">
+        <v>4</v>
+      </c>
+      <c r="G104" t="n">
+        <v>5</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -4301,25 +4355,17 @@
           <t>Wizards</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D105" t="n">
+        <v>3</v>
+      </c>
+      <c r="E105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" t="n">
+        <v>5</v>
+      </c>
+      <c r="G105" t="n">
+        <v>-1</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -4453,25 +4499,17 @@
           <t>Titan</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D109" t="n">
+        <v>5</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" t="n">
+        <v>3</v>
+      </c>
+      <c r="G109" t="n">
+        <v>31</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -4491,19 +4529,25 @@
           <t>hoorai</t>
         </is>
       </c>
-      <c r="D110" t="n">
-        <v>1</v>
-      </c>
-      <c r="E110" t="n">
-        <v>1</v>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G110" t="n">
-        <v>8</v>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -4561,25 +4605,17 @@
           <t>Verdant</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D112" t="n">
+        <v>7</v>
+      </c>
+      <c r="E112" t="n">
+        <v>6</v>
+      </c>
+      <c r="F112" t="n">
+        <v>3</v>
+      </c>
+      <c r="G112" t="n">
+        <v>56</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
update 3.2 (americas rmr b)
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -553,25 +553,17 @@
           <t>Liquid</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>52</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -895,17 +887,25 @@
           <t>Legacy</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" t="n">
-        <v>5</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -925,25 +925,17 @@
           <t>MIBR</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>8</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1533,25 +1525,17 @@
           <t>SK</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" t="n">
+        <v>5</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1647,19 +1631,25 @@
           <t>Iluminar</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>7</v>
-      </c>
-      <c r="E33" t="n">
-        <v>6</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G33" t="n">
-        <v>66</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2254,14 +2244,20 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" t="n">
-        <v>4</v>
-      </c>
-      <c r="G49" t="n">
-        <v>7</v>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2357,25 +2353,17 @@
           <t>ECSTATIC</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>4</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-4</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2395,17 +2383,25 @@
           <t>RED Canids</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>5</v>
-      </c>
-      <c r="E53" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" t="n">
-        <v>4</v>
-      </c>
-      <c r="G53" t="n">
-        <v>24</v>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2501,25 +2497,17 @@
           <t>Elevate</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D56" t="n">
+        <v>8</v>
+      </c>
+      <c r="E56" t="n">
+        <v>4</v>
+      </c>
+      <c r="F56" t="n">
+        <v>4</v>
+      </c>
+      <c r="G56" t="n">
+        <v>51</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -2653,25 +2641,17 @@
           <t>Orbit</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D60" t="n">
+        <v>6</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>4</v>
+      </c>
+      <c r="G60" t="n">
+        <v>35</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -2995,25 +2975,17 @@
           <t>Bounty Hunters</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>2</v>
+      </c>
+      <c r="G69" t="n">
+        <v>40</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -4325,17 +4297,25 @@
           <t>Bad News Eagles</t>
         </is>
       </c>
-      <c r="D104" t="n">
-        <v>3</v>
-      </c>
-      <c r="E104" t="n">
-        <v>0</v>
-      </c>
-      <c r="F104" t="n">
-        <v>4</v>
-      </c>
-      <c r="G104" t="n">
-        <v>5</v>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -4355,17 +4335,25 @@
           <t>Wizards</t>
         </is>
       </c>
-      <c r="D105" t="n">
-        <v>3</v>
-      </c>
-      <c r="E105" t="n">
-        <v>0</v>
-      </c>
-      <c r="F105" t="n">
-        <v>5</v>
-      </c>
-      <c r="G105" t="n">
-        <v>-1</v>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -4499,17 +4487,25 @@
           <t>Titan</t>
         </is>
       </c>
-      <c r="D109" t="n">
-        <v>5</v>
-      </c>
-      <c r="E109" t="n">
-        <v>0</v>
-      </c>
-      <c r="F109" t="n">
-        <v>3</v>
-      </c>
-      <c r="G109" t="n">
-        <v>31</v>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -4567,25 +4563,17 @@
           <t>GODSENT</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D111" t="n">
+        <v>3</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="n">
+        <v>5</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -4605,17 +4593,25 @@
           <t>Verdant</t>
         </is>
       </c>
-      <c r="D112" t="n">
-        <v>7</v>
-      </c>
-      <c r="E112" t="n">
-        <v>6</v>
-      </c>
-      <c r="F112" t="n">
-        <v>3</v>
-      </c>
-      <c r="G112" t="n">
-        <v>56</v>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
New System for Add Points
update 3.8
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -1280,14 +1280,20 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G23" t="n">
-        <v>-12</v>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -2794,14 +2800,20 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E63" t="n">
-        <v>0</v>
-      </c>
-      <c r="F63" t="n">
-        <v>2</v>
-      </c>
-      <c r="G63" t="n">
-        <v>-2</v>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -3087,17 +3099,25 @@
           <t>Spirit Academy</t>
         </is>
       </c>
-      <c r="D71" t="n">
-        <v>4</v>
-      </c>
-      <c r="E71" t="n">
-        <v>0</v>
-      </c>
-      <c r="F71" t="n">
-        <v>5</v>
-      </c>
-      <c r="G71" t="n">
-        <v>8</v>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -3231,17 +3251,25 @@
           <t>PARIVISION</t>
         </is>
       </c>
-      <c r="D75" t="n">
-        <v>7</v>
-      </c>
-      <c r="E75" t="n">
-        <v>4</v>
-      </c>
-      <c r="F75" t="n">
-        <v>1</v>
-      </c>
-      <c r="G75" t="n">
-        <v>60</v>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -3641,17 +3669,25 @@
           <t>Chinggis Warrios</t>
         </is>
       </c>
-      <c r="D86" t="n">
-        <v>6</v>
-      </c>
-      <c r="E86" t="n">
-        <v>0</v>
-      </c>
-      <c r="F86" t="n">
-        <v>5</v>
-      </c>
-      <c r="G86" t="n">
-        <v>26</v>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -3747,17 +3783,25 @@
           <t>MenaceGG</t>
         </is>
       </c>
-      <c r="D89" t="n">
-        <v>4</v>
-      </c>
-      <c r="E89" t="n">
-        <v>0</v>
-      </c>
-      <c r="F89" t="n">
-        <v>4</v>
-      </c>
-      <c r="G89" t="n">
-        <v>13</v>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -4081,17 +4125,25 @@
           <t>Nemiga</t>
         </is>
       </c>
-      <c r="D98" t="n">
-        <v>7</v>
-      </c>
-      <c r="E98" t="n">
-        <v>4</v>
-      </c>
-      <c r="F98" t="n">
-        <v>3</v>
-      </c>
-      <c r="G98" t="n">
-        <v>48</v>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -4529,17 +4581,25 @@
           <t>hoorai</t>
         </is>
       </c>
-      <c r="D110" t="n">
-        <v>5</v>
-      </c>
-      <c r="E110" t="n">
-        <v>0</v>
-      </c>
-      <c r="F110" t="n">
-        <v>2</v>
-      </c>
-      <c r="G110" t="n">
-        <v>40</v>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix - America OQ
update 6.1
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -553,25 +553,17 @@
           <t>Liquid</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>63</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -596,20 +588,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-5</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -857,25 +843,17 @@
           <t>FURIA</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -933,25 +911,17 @@
           <t>MIBR</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>8</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1166,14 +1136,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" t="n">
-        <v>-5</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1535,25 +1511,17 @@
           <t>SK</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" t="n">
+        <v>5</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1578,20 +1546,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-5</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1649,17 +1611,25 @@
           <t>Iluminar</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>8</v>
-      </c>
-      <c r="E33" t="n">
-        <v>7</v>
-      </c>
-      <c r="F33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" t="n">
-        <v>80</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2216,20 +2186,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-5</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -2249,25 +2213,17 @@
           <t>M80</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>4</v>
+      </c>
+      <c r="G49" t="n">
+        <v>7</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2363,25 +2319,17 @@
           <t>ECSTATIC</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>4</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-4</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2401,25 +2349,17 @@
           <t>RED Canids</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D53" t="n">
+        <v>6</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>6</v>
+      </c>
+      <c r="G53" t="n">
+        <v>22</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2444,20 +2384,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="n">
+        <v>-5</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2482,14 +2416,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" t="n">
-        <v>1</v>
-      </c>
-      <c r="G55" t="n">
-        <v>-5</v>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -2509,17 +2449,25 @@
           <t>Elevate</t>
         </is>
       </c>
-      <c r="D56" t="n">
-        <v>11</v>
-      </c>
-      <c r="E56" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" t="n">
-        <v>8</v>
-      </c>
-      <c r="G56" t="n">
-        <v>56</v>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -2653,25 +2601,17 @@
           <t>Orbit</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D60" t="n">
+        <v>7</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>6</v>
+      </c>
+      <c r="G60" t="n">
+        <v>33</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -2848,20 +2788,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-5</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -2995,25 +2929,17 @@
           <t>Bounty Hunters</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D69" t="n">
+        <v>9</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>8</v>
+      </c>
+      <c r="G69" t="n">
+        <v>45</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -3722,20 +3648,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" t="n">
+        <v>-5</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -4406,20 +4326,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" t="n">
+        <v>-5</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -4482,20 +4396,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" t="n">
+        <v>-5</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -4515,25 +4423,17 @@
           <t>Titan</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D109" t="n">
+        <v>10</v>
+      </c>
+      <c r="E109" t="n">
+        <v>3</v>
+      </c>
+      <c r="F109" t="n">
+        <v>7</v>
+      </c>
+      <c r="G109" t="n">
+        <v>55</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -4591,25 +4491,17 @@
           <t>GODSENT</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D111" t="n">
+        <v>3</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="n">
+        <v>5</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -4672,20 +4564,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="n">
+        <v>1</v>
+      </c>
+      <c r="G113" t="n">
+        <v>-5</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Final Fix - Asia Teams
update 7
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -477,19 +477,25 @@
           <t>Vitality</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>8</v>
-      </c>
-      <c r="E2" t="n">
-        <v>8</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>92</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -509,17 +515,25 @@
           <t>Astralis</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-12</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -615,17 +629,25 @@
           <t>Heroic</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" t="n">
-        <v>57</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -683,17 +705,25 @@
           <t>FaZe</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4</v>
-      </c>
-      <c r="G8" t="n">
-        <v>15</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -751,17 +781,25 @@
           <t>ENCE</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" t="n">
-        <v>5</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -933,25 +971,17 @@
           <t>Natus Vincere</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="n">
+        <v>72</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -971,17 +1001,25 @@
           <t>MOUZ</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>3</v>
-      </c>
-      <c r="G16" t="n">
-        <v>-7</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-7</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1001,17 +1039,25 @@
           <t>G2</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>7</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>8</v>
-      </c>
-      <c r="G17" t="n">
-        <v>18</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1145,25 +1191,17 @@
           <t>Virtus.pro</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-4</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1183,25 +1221,17 @@
           <t>Spirit</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="n">
+        <v>55</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1221,25 +1251,17 @@
           <t>Entropiq</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-12</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1259,17 +1281,25 @@
           <t>Copenhagen Flames</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>15</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>5</v>
-      </c>
-      <c r="G24" t="n">
-        <v>133</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1327,17 +1357,25 @@
           <t>iBUYPOWER</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>4</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="n">
-        <v>4</v>
-      </c>
-      <c r="G26" t="n">
-        <v>15</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1369,12 +1407,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1395,17 +1433,25 @@
           <t>Dignitas</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>3</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="n">
-        <v>4</v>
-      </c>
-      <c r="G28" t="n">
-        <v>4</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1425,17 +1471,25 @@
           <t>Cloud9</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>10</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="n">
-        <v>8</v>
-      </c>
-      <c r="G29" t="n">
-        <v>45</v>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1607,17 +1661,25 @@
           <t>Falcons</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>6</v>
-      </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="n">
-        <v>3</v>
-      </c>
-      <c r="G34" t="n">
-        <v>39</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1649,12 +1711,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1725,12 +1787,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1751,17 +1813,25 @@
           <t>Nexus</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>4</v>
-      </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="n">
-        <v>4</v>
-      </c>
-      <c r="G38" t="n">
-        <v>13</v>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -1793,12 +1863,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1907,12 +1977,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -1971,17 +2041,25 @@
           <t>Rebels</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>10</v>
-      </c>
-      <c r="E44" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" t="n">
-        <v>7</v>
-      </c>
-      <c r="G44" t="n">
-        <v>54</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2001,17 +2079,25 @@
           <t>Eternal Fire</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>13</v>
-      </c>
-      <c r="E45" t="n">
-        <v>4</v>
-      </c>
-      <c r="F45" t="n">
-        <v>6</v>
-      </c>
-      <c r="G45" t="n">
-        <v>85</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2036,14 +2122,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" t="n">
-        <v>-5</v>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2068,14 +2160,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E47" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" t="n">
-        <v>3</v>
-      </c>
-      <c r="G47" t="n">
-        <v>-15</v>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>-15</t>
+        </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2171,17 +2269,25 @@
           <t>Wildcard</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" t="n">
-        <v>4</v>
-      </c>
-      <c r="G50" t="n">
-        <v>-12</v>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -2201,25 +2307,17 @@
           <t>BESTIA</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>8</v>
+      </c>
+      <c r="G51" t="n">
+        <v>40</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -2467,25 +2565,17 @@
           <t>Underground</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D58" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>4</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-3</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -2619,25 +2709,17 @@
           <t>Homyno</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D62" t="n">
+        <v>4</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>4</v>
+      </c>
+      <c r="G62" t="n">
+        <v>15</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -2657,25 +2739,17 @@
           <t>Take Flyte</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>4</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-4</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -2783,12 +2857,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -2821,12 +2895,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -2844,28 +2918,20 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Team Solid</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>Solid</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>4</v>
+      </c>
+      <c r="G68" t="n">
+        <v>15</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -2963,7 +3029,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2973,12 +3039,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3011,12 +3077,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3037,25 +3103,17 @@
           <t>The MongolZ</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D73" t="n">
+        <v>13</v>
+      </c>
+      <c r="E73" t="n">
+        <v>2</v>
+      </c>
+      <c r="F73" t="n">
+        <v>6</v>
+      </c>
+      <c r="G73" t="n">
+        <v>86</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -3115,22 +3173,22 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3163,12 +3221,12 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3189,25 +3247,17 @@
           <t>VP.Prodigy</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D77" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" t="n">
+        <v>4</v>
+      </c>
+      <c r="G77" t="n">
+        <v>-3</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -3229,7 +3279,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3239,12 +3289,12 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>41</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3277,12 +3327,12 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3305,7 +3355,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3315,12 +3365,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>38</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3353,12 +3403,12 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3391,12 +3441,12 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3417,25 +3467,17 @@
           <t>TYLOO</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D83" t="n">
+        <v>9</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>8</v>
+      </c>
+      <c r="G83" t="n">
+        <v>42</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -3467,12 +3509,12 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -3505,12 +3547,12 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -3533,7 +3575,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3543,12 +3585,12 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>16</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -3581,12 +3623,12 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -3645,25 +3687,17 @@
           <t>MenaceGG</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D89" t="n">
+        <v>4</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" t="n">
+        <v>4</v>
+      </c>
+      <c r="G89" t="n">
+        <v>13</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -3695,12 +3729,12 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -3733,12 +3767,12 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -3759,25 +3793,17 @@
           <t>Aravt</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D92" t="n">
+        <v>3</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="n">
+        <v>4</v>
+      </c>
+      <c r="G92" t="n">
+        <v>5</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -3809,12 +3835,12 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -3835,25 +3861,17 @@
           <t>True Rippers</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D94" t="n">
+        <v>3</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="n">
+        <v>5</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -3875,7 +3893,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -3885,12 +3903,12 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -3923,12 +3941,12 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -3961,12 +3979,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -3989,7 +4007,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -3999,12 +4017,12 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>80</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4037,12 +4055,12 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4075,12 +4093,12 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4101,25 +4119,17 @@
           <t>Onyx Ravens</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D101" t="n">
+        <v>11</v>
+      </c>
+      <c r="E101" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" t="n">
+        <v>9</v>
+      </c>
+      <c r="G101" t="n">
+        <v>48</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -4151,12 +4161,12 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-5</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4174,7 +4184,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Reason Gaming</t>
+          <t>Reason</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -4189,12 +4199,12 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-15</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4443,25 +4453,17 @@
           <t>hoorai</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="D110" t="n">
+        <v>6</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" t="n">
+        <v>6</v>
+      </c>
+      <c r="G110" t="n">
+        <v>28</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -4972,7 +4974,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Team Kinguin</t>
+          <t>Kinguin</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">

</xml_diff>

<commit_message>
clean up repo, finalize README, fix minor bug
- Finalize README;
- Add .gitignore for __pycache__ and remove already-tracked files
- Little fix in db_manipulation.py comment
- Removed not essential packages from requirements.txt
</commit_message>
<xml_diff>
--- a/hltv.xlsx
+++ b/hltv.xlsx
@@ -464,27 +464,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
     </row>

</xml_diff>